<commit_message>
fix(attendance): clean sample excel columns and relocate sample download button
</commit_message>
<xml_diff>
--- a/frontend/public/templates/attendance_sample_record.xlsx
+++ b/frontend/public/templates/attendance_sample_record.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="record" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,23 +28,20 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00111827"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="004B5563"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001F2937"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00111827"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -62,7 +59,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -84,72 +81,6 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D1D5DB"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D1D5DB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D1D5DB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00D1D5DB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00D1D5DB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D1D5DB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D1D5DB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D1D5DB"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -157,13 +88,11 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -535,346 +464,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:M9"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="D1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>record</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="D2" s="1" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>unit: Syaco    date from: 2026-08-03 to 2026-08-03 23:59</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>user_no</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>user_lname</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>user_depname</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>sj</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>fx</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>iden</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>healthstatus</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>body_temp</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>dev_serial</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>lx</t>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>รหัส</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>ชื่อ-สกุล</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>แผนก-ฝ่าย.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>วันที่-เวลา</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>สถานะ</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ลงเวลาด้วย</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>การตรวจอุณหภูมิ</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>เครื่อง</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>ประมวลผล</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>รหัส</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ชื่อ-สกุล</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>แผนก-ฝ่าย.</t>
-        </is>
-      </c>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>วันที่-เวลา</t>
+          <t>อุณหภูมิ</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>สถานะ</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>ลงเวลาด้วย</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>การตรวจอุณหภูมิ</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>เครื่อง</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>ประมวลผล</t>
-        </is>
-      </c>
+          <t>องศา</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
     </row>
-    <row r="5">
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>อุณหภูมิ</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>องศา</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>100001</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>สมชาย</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Syaco</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:49:12</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Attendance</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
     </row>
-    <row r="6">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>100001</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>สมชาย</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Syaco</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>2026-08-03 12:54:49</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Attendance</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>EARLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
           <t>100001</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>สมชาย</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Syaco</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-03 09:49:12</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03 13:04:08</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>l</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Attendance</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>IN</t>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>INVALID</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="D7" s="5" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>100001</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>สมชาย</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Syaco</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-03 12:54:49</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03 18:08:31</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>l</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Attendance</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>EARLY</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>100001</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>สมชาย</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Syaco</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-03 13:04:08</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
       <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>Attendance</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>INVALID</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>100001</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>สมชาย</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Syaco</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-03 18:08:31</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>Attendance</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
@@ -882,15 +755,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="G3:H3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>